<commit_message>
ZGZGST-743 指令管理-银行间指令-银行间买断式回购指令画面，导入报错【No message found under code 'EtrFund003.chlId' for locale 'zh_CN'.】
</commit_message>
<xml_diff>
--- a/tams-invest-parent/tams-invest-entrust/src/main/resources/tpl/EtrBoutRepo003MTM.xlsx
+++ b/tams-invest-parent/tams-invest-entrust/src/main/resources/tpl/EtrBoutRepo003MTM.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9303"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="60" windowWidth="20730" windowHeight="11700"/>
+    <workbookView xWindow="0" yWindow="60" windowWidth="20736" windowHeight="11700"/>
   </bookViews>
   <sheets>
     <sheet name="数据" sheetId="1" r:id="rId1"/>
@@ -348,7 +348,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -356,9 +356,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -451,10 +448,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="373737"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr val="window" lastClr="CCEDC7"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -709,17 +706,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:V101"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <dimension ref="A1:V3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="12" width="14.625" customWidth="1"/>
-    <col min="13" max="13" width="22.625" customWidth="1"/>
-    <col min="14" max="14" width="15.625" customWidth="1"/>
-    <col min="15" max="19" width="14.625" customWidth="1"/>
-    <col min="20" max="20" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="12" width="14.6640625" customWidth="1"/>
+    <col min="13" max="13" width="22.6640625" customWidth="1"/>
+    <col min="14" max="14" width="15.6640625" customWidth="1"/>
+    <col min="15" max="19" width="14.6640625" customWidth="1"/>
+    <col min="20" max="20" width="10.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -787,309 +784,13 @@
         <v>76</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
-      <c r="R2" s="3"/>
-    </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.15">
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
-      <c r="R3" s="3"/>
-    </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="R4" s="3"/>
-    </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="R5" s="3"/>
-    </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="R6" s="3"/>
-    </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="R7" s="3"/>
-    </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="R8" s="3"/>
-    </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="R9" s="3"/>
-    </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="R10" s="3"/>
-    </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="R11" s="3"/>
-    </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="R12" s="3"/>
-    </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="R13" s="3"/>
-    </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="R14" s="3"/>
-    </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="R15" s="3"/>
-    </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="R16" s="3"/>
-    </row>
-    <row r="17" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R17" s="3"/>
-    </row>
-    <row r="18" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R18" s="3"/>
-    </row>
-    <row r="19" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R19" s="3"/>
-    </row>
-    <row r="20" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R20" s="3"/>
-    </row>
-    <row r="21" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R21" s="3"/>
-    </row>
-    <row r="22" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R22" s="3"/>
-    </row>
-    <row r="23" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R23" s="3"/>
-    </row>
-    <row r="24" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R24" s="3"/>
-    </row>
-    <row r="25" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R25" s="3"/>
-    </row>
-    <row r="26" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R26" s="3"/>
-    </row>
-    <row r="27" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R27" s="3"/>
-    </row>
-    <row r="28" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R28" s="3"/>
-    </row>
-    <row r="29" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R29" s="3"/>
-    </row>
-    <row r="30" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R30" s="3"/>
-    </row>
-    <row r="31" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R31" s="3"/>
-    </row>
-    <row r="32" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R32" s="3"/>
-    </row>
-    <row r="33" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R33" s="3"/>
-    </row>
-    <row r="34" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R34" s="3"/>
-    </row>
-    <row r="35" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R35" s="3"/>
-    </row>
-    <row r="36" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R36" s="3"/>
-    </row>
-    <row r="37" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R37" s="3"/>
-    </row>
-    <row r="38" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R38" s="3"/>
-    </row>
-    <row r="39" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R39" s="3"/>
-    </row>
-    <row r="40" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R40" s="3"/>
-    </row>
-    <row r="41" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R41" s="3"/>
-    </row>
-    <row r="42" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R42" s="3"/>
-    </row>
-    <row r="43" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R43" s="3"/>
-    </row>
-    <row r="44" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R44" s="3"/>
-    </row>
-    <row r="45" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R45" s="3"/>
-    </row>
-    <row r="46" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R46" s="3"/>
-    </row>
-    <row r="47" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R47" s="3"/>
-    </row>
-    <row r="48" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R48" s="3"/>
-    </row>
-    <row r="49" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R49" s="3"/>
-    </row>
-    <row r="50" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R50" s="3"/>
-    </row>
-    <row r="51" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R51" s="3"/>
-    </row>
-    <row r="52" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R52" s="3"/>
-    </row>
-    <row r="53" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R53" s="3"/>
-    </row>
-    <row r="54" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R54" s="3"/>
-    </row>
-    <row r="55" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R55" s="3"/>
-    </row>
-    <row r="56" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R56" s="3"/>
-    </row>
-    <row r="57" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R57" s="3"/>
-    </row>
-    <row r="58" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R58" s="3"/>
-    </row>
-    <row r="59" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R59" s="3"/>
-    </row>
-    <row r="60" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R60" s="3"/>
-    </row>
-    <row r="61" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R61" s="3"/>
-    </row>
-    <row r="62" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R62" s="3"/>
-    </row>
-    <row r="63" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R63" s="3"/>
-    </row>
-    <row r="64" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R64" s="3"/>
-    </row>
-    <row r="65" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R65" s="3"/>
-    </row>
-    <row r="66" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R66" s="3"/>
-    </row>
-    <row r="67" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R67" s="3"/>
-    </row>
-    <row r="68" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R68" s="3"/>
-    </row>
-    <row r="69" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R69" s="3"/>
-    </row>
-    <row r="70" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R70" s="3"/>
-    </row>
-    <row r="71" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R71" s="3"/>
-    </row>
-    <row r="72" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R72" s="3"/>
-    </row>
-    <row r="73" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R73" s="3"/>
-    </row>
-    <row r="74" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R74" s="3"/>
-    </row>
-    <row r="75" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R75" s="3"/>
-    </row>
-    <row r="76" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R76" s="3"/>
-    </row>
-    <row r="77" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R77" s="3"/>
-    </row>
-    <row r="78" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R78" s="3"/>
-    </row>
-    <row r="79" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R79" s="3"/>
-    </row>
-    <row r="80" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R80" s="3"/>
-    </row>
-    <row r="81" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R81" s="3"/>
-    </row>
-    <row r="82" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R82" s="3"/>
-    </row>
-    <row r="83" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R83" s="3"/>
-    </row>
-    <row r="84" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R84" s="3"/>
-    </row>
-    <row r="85" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R85" s="3"/>
-    </row>
-    <row r="86" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R86" s="3"/>
-    </row>
-    <row r="87" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R87" s="3"/>
-    </row>
-    <row r="88" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R88" s="3"/>
-    </row>
-    <row r="89" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R89" s="3"/>
-    </row>
-    <row r="90" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R90" s="3"/>
-    </row>
-    <row r="91" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R91" s="3"/>
-    </row>
-    <row r="92" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R92" s="3"/>
-    </row>
-    <row r="93" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R93" s="3"/>
-    </row>
-    <row r="94" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R94" s="3"/>
-    </row>
-    <row r="95" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R95" s="3"/>
-    </row>
-    <row r="96" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R96" s="3"/>
-    </row>
-    <row r="97" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R97" s="3"/>
-    </row>
-    <row r="98" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R98" s="3"/>
-    </row>
-    <row r="99" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R99" s="3"/>
-    </row>
-    <row r="100" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R100" s="3"/>
-    </row>
-    <row r="101" spans="18:18" x14ac:dyDescent="0.15">
-      <c r="R101" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -1111,7 +812,7 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>Sheet1!$A$2:$A$31</xm:f>
@@ -1124,6 +825,12 @@
           </x14:formula1>
           <xm:sqref>Q2:Q101</xm:sqref>
         </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>Sheet1!$C$2:$C$13</xm:f>
+          </x14:formula1>
+          <xm:sqref>R2:R1048576</xm:sqref>
+        </x14:dataValidation>
       </x14:dataValidations>
     </ext>
   </extLst>
@@ -1133,14 +840,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C31"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.375" customWidth="1"/>
-    <col min="2" max="2" width="20.5" customWidth="1"/>
-    <col min="3" max="3" width="17.5" customWidth="1"/>
+    <col min="1" max="1" width="23.33203125" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" customWidth="1"/>
+    <col min="3" max="3" width="17.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -1151,7 +858,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1162,7 +869,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>22</v>
       </c>
@@ -1173,7 +880,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>23</v>
       </c>
@@ -1184,7 +891,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -1195,7 +902,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -1206,7 +913,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>26</v>
       </c>
@@ -1217,7 +924,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>27</v>
       </c>
@@ -1228,7 +935,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>28</v>
       </c>
@@ -1239,7 +946,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>29</v>
       </c>
@@ -1250,7 +957,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -1261,7 +968,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -1272,7 +979,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -1280,92 +987,92 @@
         <v>75</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>50</v>
       </c>

</xml_diff>